<commit_message>
Rename of tests + script1 assertion implemented
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\CMTF_AOADMM_refactor\examples\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\CMTF_AOADMM_refactor\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E9FD80-A970-4C91-8146-9B24FDA3A1F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BD0B9C7-1BF4-4333-B643-9EF0172CB272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="27">
   <si>
     <t>Example script number</t>
   </si>
@@ -102,6 +102,21 @@
   </si>
   <si>
     <t>A: 1</t>
+  </si>
+  <si>
+    <t>Correct</t>
+  </si>
+  <si>
+    <t>Refactor</t>
+  </si>
+  <si>
+    <t>Broken</t>
+  </si>
+  <si>
+    <t>Correct?</t>
+  </si>
+  <si>
+    <t>Fig different?</t>
   </si>
 </sst>
 </file>
@@ -123,7 +138,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -133,6 +148,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -149,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -158,10 +185,15 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -496,7 +528,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6001F213-F06F-43A9-9C65-6A6D4326F486}">
-  <dimension ref="B2:R19"/>
+  <dimension ref="B2:U19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19.36328125" bestFit="1" customWidth="1"/>
@@ -509,9 +541,10 @@
     <col min="12" max="13" width="7.1796875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="7.36328125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.1796875" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
@@ -527,31 +560,31 @@
       <c r="F2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="2" t="s">
         <v>16</v>
       </c>
       <c r="Q2" s="2" t="s">
@@ -560,8 +593,11 @@
       <c r="R2" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="3" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="T2" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B3" s="2">
         <v>1</v>
       </c>
@@ -577,35 +613,38 @@
       <c r="F3" s="2">
         <v>0</v>
       </c>
-      <c r="G3" s="4">
-        <v>0</v>
-      </c>
-      <c r="H3" s="4">
+      <c r="G3" s="2">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2">
         <v>100</v>
       </c>
-      <c r="I3" s="4">
+      <c r="I3" s="2">
         <v>100</v>
       </c>
-      <c r="J3" s="4">
+      <c r="J3" s="2">
         <v>1</v>
       </c>
       <c r="K3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="2">
         <v>1</v>
       </c>
-      <c r="M3" s="4">
+      <c r="M3" s="2">
         <v>1</v>
       </c>
-      <c r="N3" s="4">
+      <c r="N3" s="2">
         <v>1</v>
       </c>
-      <c r="O3" s="5" t="s">
+      <c r="O3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="T3" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
@@ -621,33 +660,36 @@
       <c r="F4" s="2">
         <v>0</v>
       </c>
-      <c r="G4" s="4">
-        <v>0</v>
-      </c>
-      <c r="H4" s="4">
+      <c r="G4" s="2">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2">
         <v>79.909700000000001</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="2">
         <v>79.275899999999993</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="2">
         <v>0.99399999999999999</v>
       </c>
       <c r="K4" s="3"/>
-      <c r="L4" s="4">
+      <c r="L4" s="2">
         <v>0.99560000000000004</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="2">
         <v>0.96099999999999997</v>
       </c>
-      <c r="N4" s="4">
+      <c r="N4" s="2">
         <v>0.998</v>
       </c>
-      <c r="O4" s="5" t="s">
+      <c r="O4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="T4" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B5" s="2">
         <v>2</v>
       </c>
@@ -663,33 +705,36 @@
       <c r="F5" s="2">
         <v>0</v>
       </c>
-      <c r="G5" s="4">
-        <v>0</v>
-      </c>
-      <c r="H5" s="4">
+      <c r="G5" s="2">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2">
         <v>82.112099999999998</v>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="2">
         <v>80.918099999999995</v>
       </c>
-      <c r="J5" s="4">
+      <c r="J5" s="2">
         <v>0.92290000000000005</v>
       </c>
       <c r="K5" s="3"/>
-      <c r="L5" s="4">
+      <c r="L5" s="2">
         <v>0.98140000000000005</v>
       </c>
-      <c r="M5" s="4">
+      <c r="M5" s="2">
         <v>0.93840000000000001</v>
       </c>
-      <c r="N5" s="4">
+      <c r="N5" s="2">
         <v>0.99470000000000003</v>
       </c>
-      <c r="O5" s="5" t="s">
+      <c r="O5" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="T5" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B6" s="2">
         <v>3</v>
       </c>
@@ -705,29 +750,32 @@
       <c r="F6" s="2">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="G6" s="4">
-        <v>0</v>
-      </c>
-      <c r="H6" s="4">
+      <c r="G6" s="2">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2">
         <v>96.162800000000004</v>
       </c>
-      <c r="I6" s="4">
+      <c r="I6" s="2">
         <v>96.4923</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="2">
         <v>0.99870000000000003</v>
       </c>
-      <c r="K6" s="4">
+      <c r="K6" s="2">
         <v>0.97350000000000003</v>
       </c>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
-      <c r="O6" s="5" t="s">
+      <c r="O6" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="7" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="T6" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B7" s="2">
         <v>4</v>
       </c>
@@ -743,29 +791,32 @@
       <c r="F7" s="2">
         <v>0</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="2">
         <v>0</v>
       </c>
       <c r="H7" s="3"/>
-      <c r="I7" s="4">
+      <c r="I7" s="2">
         <v>96.438000000000002</v>
       </c>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
-      <c r="L7" s="4">
+      <c r="L7" s="2">
         <v>1</v>
       </c>
-      <c r="M7" s="4">
+      <c r="M7" s="2">
         <v>0.99419999999999997</v>
       </c>
-      <c r="N7" s="4">
+      <c r="N7" s="2">
         <v>1</v>
       </c>
-      <c r="O7" s="5" t="s">
+      <c r="O7" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="T7" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B8" s="2">
         <v>5</v>
       </c>
@@ -781,29 +832,32 @@
       <c r="F8" s="2">
         <v>0</v>
       </c>
-      <c r="G8" s="4">
-        <v>0</v>
-      </c>
-      <c r="H8" s="4">
+      <c r="G8" s="2">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2">
         <v>96.170500000000004</v>
       </c>
-      <c r="I8" s="4">
+      <c r="I8" s="2">
         <v>96.153400000000005</v>
       </c>
-      <c r="J8" s="4">
+      <c r="J8" s="2">
         <v>0.99890000000000001</v>
       </c>
-      <c r="K8" s="4">
+      <c r="K8" s="2">
         <v>0.99960000000000004</v>
       </c>
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
-      <c r="O8" s="5" t="s">
+      <c r="O8" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="T8" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B9" s="2">
         <v>6</v>
       </c>
@@ -819,25 +873,25 @@
       <c r="F9" s="2">
         <v>0</v>
       </c>
-      <c r="G9" s="4">
-        <v>0</v>
-      </c>
-      <c r="H9" s="4">
+      <c r="G9" s="2">
+        <v>0</v>
+      </c>
+      <c r="H9" s="2">
         <v>96.127499999999998</v>
       </c>
-      <c r="I9" s="4">
+      <c r="I9" s="2">
         <v>96.408299999999997</v>
       </c>
-      <c r="J9" s="4">
+      <c r="J9" s="2">
         <v>0.99670000000000003</v>
       </c>
-      <c r="K9" s="4">
+      <c r="K9" s="2">
         <v>0.98299999999999998</v>
       </c>
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
-      <c r="O9" s="5" t="s">
+      <c r="O9" t="s">
         <v>14</v>
       </c>
       <c r="Q9">
@@ -846,8 +900,11 @@
       <c r="R9">
         <v>0.98309999999999997</v>
       </c>
-    </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="T9" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B10" s="2">
         <v>7</v>
       </c>
@@ -863,29 +920,32 @@
       <c r="F10" s="2">
         <v>0</v>
       </c>
-      <c r="G10" s="4">
-        <v>0</v>
-      </c>
-      <c r="H10" s="4">
+      <c r="G10" s="2">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2">
         <v>89.872200000000007</v>
       </c>
-      <c r="I10" s="4">
+      <c r="I10" s="2">
         <v>87.011499999999998</v>
       </c>
-      <c r="J10" s="4">
+      <c r="J10" s="2">
         <v>0.99450000000000005</v>
       </c>
-      <c r="K10" s="4">
+      <c r="K10" s="2">
         <v>0.95040000000000002</v>
       </c>
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
-      <c r="O10" s="5" t="s">
+      <c r="O10" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="T10" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B11" s="2">
         <v>8</v>
       </c>
@@ -901,23 +961,26 @@
       <c r="F11" s="2">
         <v>0</v>
       </c>
-      <c r="G11" s="4">
-        <v>0</v>
-      </c>
-      <c r="H11" s="4">
+      <c r="G11" s="2">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2">
         <v>96.433899999999994</v>
       </c>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="O11" s="5" t="s">
+      <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+      <c r="O11" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="T11" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B12" s="2">
         <v>9</v>
       </c>
@@ -933,32 +996,38 @@
       <c r="F12" s="2">
         <v>1.503E-3</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="2">
         <v>3.5500000000000001E-4</v>
       </c>
       <c r="H12" s="3"/>
-      <c r="I12" s="4">
+      <c r="I12" s="2">
         <v>95.735299999999995</v>
       </c>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
-      <c r="L12" s="4">
+      <c r="L12" s="2">
         <v>0.99980000000000002</v>
       </c>
-      <c r="M12" s="4">
+      <c r="M12" s="2">
         <v>0.98170000000000002</v>
       </c>
-      <c r="N12" s="4">
+      <c r="N12" s="2">
         <v>0.99970000000000003</v>
       </c>
-      <c r="O12" s="5" t="s">
+      <c r="O12" t="s">
         <v>20</v>
       </c>
       <c r="Q12" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="T12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="U12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B13" s="2">
         <v>10</v>
       </c>
@@ -991,8 +1060,14 @@
       <c r="O13" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="T13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="U13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B14" s="2">
         <v>11</v>
       </c>
@@ -1029,8 +1104,11 @@
       <c r="O14" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="T14" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -1045,7 +1123,7 @@
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
     </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>

</xml_diff>

<commit_message>
Assertions added to all tests of examples
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\CMTF_AOADMM_refactor\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BD0B9C7-1BF4-4333-B643-9EF0172CB272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC9E7E31-12FE-41C6-91B8-6E8FEFE784BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -176,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -189,9 +189,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -529,22 +526,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6001F213-F06F-43A9-9C65-6A6D4326F486}">
   <dimension ref="B2:U19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.08984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="6.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.36328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.1796875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.140625" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:21" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
@@ -597,7 +594,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="2:21" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B3" s="2">
         <v>1</v>
       </c>
@@ -644,7 +641,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="2:21" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
@@ -689,7 +686,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="2:21" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B5" s="2">
         <v>2</v>
       </c>
@@ -734,7 +731,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="2:21" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B6" s="2">
         <v>3</v>
       </c>
@@ -775,7 +772,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="2:21" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
         <v>4</v>
       </c>
@@ -816,7 +813,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="2:21" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
         <v>5</v>
       </c>
@@ -857,7 +854,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="2:21" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B9" s="2">
         <v>6</v>
       </c>
@@ -904,7 +901,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="2:21" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
         <v>7</v>
       </c>
@@ -945,7 +942,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="2:21" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B11" s="2">
         <v>8</v>
       </c>
@@ -970,9 +967,15 @@
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
+      <c r="L11" s="2">
+        <v>0.999</v>
+      </c>
+      <c r="M11" s="2">
+        <v>0.98580000000000001</v>
+      </c>
+      <c r="N11" s="2">
+        <v>0.99950000000000006</v>
+      </c>
       <c r="O11" t="s">
         <v>14</v>
       </c>
@@ -980,7 +983,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="2:21" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B12" s="2">
         <v>9</v>
       </c>
@@ -1027,7 +1030,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="2:21" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B13" s="2">
         <v>10</v>
       </c>
@@ -1067,7 +1070,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="2:21" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B14" s="2">
         <v>11</v>
       </c>
@@ -1108,7 +1111,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="2:21" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -1123,7 +1126,7 @@
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
     </row>
-    <row r="16" spans="2:21" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -1138,7 +1141,7 @@
       <c r="M16" s="2"/>
       <c r="N16" s="2"/>
     </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -1153,7 +1156,7 @@
       <c r="M17" s="2"/>
       <c r="N17" s="2"/>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -1168,7 +1171,7 @@
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
     </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>

</xml_diff>

<commit_message>
Updated expected output under stable seed
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\CMTF_AOADMM_refactor\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC9E7E31-12FE-41C6-91B8-6E8FEFE784BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6181D77E-22A0-42A5-9702-15DF7ED9DC6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
@@ -95,15 +95,9 @@
     <t>FMS3</t>
   </si>
   <si>
-    <t>difficult problem!</t>
-  </si>
-  <si>
     <t>maxIterations</t>
   </si>
   <si>
-    <t>A: 1</t>
-  </si>
-  <si>
     <t>Correct</t>
   </si>
   <si>
@@ -117,6 +111,12 @@
   </si>
   <si>
     <t>Fig different?</t>
+  </si>
+  <si>
+    <t>0,000007</t>
+  </si>
+  <si>
+    <t>Run under rng(123, 'twister')</t>
   </si>
 </sst>
 </file>
@@ -138,7 +138,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -147,19 +147,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="1"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor theme="2" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -178,19 +172,17 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -525,7 +517,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6001F213-F06F-43A9-9C65-6A6D4326F486}">
-  <dimension ref="B2:U19"/>
+  <dimension ref="B1:U19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
@@ -538,63 +530,68 @@
     <col min="12" max="13" width="7.140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="7.42578125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.140625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2" t="s">
+    <row r="1" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="2:21" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="O2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="Q2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="R2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="T2" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="T2" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="2">
         <v>1</v>
       </c>
@@ -622,79 +619,77 @@
       <c r="J3" s="2">
         <v>1</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="K3" s="2"/>
       <c r="L3" s="2">
         <v>1</v>
       </c>
       <c r="M3" s="2">
-        <v>1</v>
+        <v>0.999</v>
       </c>
       <c r="N3" s="2">
         <v>1</v>
       </c>
-      <c r="O3" t="s">
+      <c r="O3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="T3" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="T3" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="2">
-        <v>0.22132299999999999</v>
+        <v>0.22369900000000001</v>
       </c>
       <c r="D4" s="2">
-        <v>0.22132199999999999</v>
-      </c>
-      <c r="E4" s="2">
-        <v>0</v>
+        <v>0.22126100000000001</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="F4" s="2">
-        <v>0</v>
+        <v>3.6000000000000001E-5</v>
       </c>
       <c r="G4" s="2">
-        <v>0</v>
+        <v>2.395E-3</v>
       </c>
       <c r="H4" s="2">
-        <v>79.909700000000001</v>
+        <v>80.028000000000006</v>
       </c>
       <c r="I4" s="2">
-        <v>79.275899999999993</v>
+        <v>79.271799999999999</v>
       </c>
       <c r="J4" s="2">
-        <v>0.99399999999999999</v>
-      </c>
-      <c r="K4" s="3"/>
+        <v>0.99760000000000004</v>
+      </c>
+      <c r="K4" s="2"/>
       <c r="L4" s="2">
-        <v>0.99560000000000004</v>
+        <v>0.99870000000000003</v>
       </c>
       <c r="M4" s="2">
-        <v>0.96099999999999997</v>
+        <v>0.94030000000000002</v>
       </c>
       <c r="N4" s="2">
-        <v>0.998</v>
-      </c>
-      <c r="O4" t="s">
-        <v>14</v>
-      </c>
-      <c r="T4" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="2:21" x14ac:dyDescent="0.25">
+        <v>0.99660000000000004</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2">
         <v>2</v>
       </c>
       <c r="C5" s="2">
-        <v>0.18401999999999999</v>
+        <v>0.18159600000000001</v>
       </c>
       <c r="D5" s="2">
-        <v>0.18401999999999999</v>
+        <v>0.18159500000000001</v>
       </c>
       <c r="E5" s="2">
         <v>0</v>
@@ -706,43 +701,43 @@
         <v>0</v>
       </c>
       <c r="H5" s="2">
-        <v>82.112099999999998</v>
+        <v>82.649000000000001</v>
       </c>
       <c r="I5" s="2">
-        <v>80.918099999999995</v>
+        <v>81.117699999999999</v>
       </c>
       <c r="J5" s="2">
-        <v>0.92290000000000005</v>
-      </c>
-      <c r="K5" s="3"/>
+        <v>0.91859999999999997</v>
+      </c>
+      <c r="K5" s="2"/>
       <c r="L5" s="2">
-        <v>0.98140000000000005</v>
+        <v>0.97509999999999997</v>
       </c>
       <c r="M5" s="2">
-        <v>0.93840000000000001</v>
+        <v>0.93130000000000002</v>
       </c>
       <c r="N5" s="2">
-        <v>0.99470000000000003</v>
-      </c>
-      <c r="O5" t="s">
+        <v>0.9909</v>
+      </c>
+      <c r="O5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="T5" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="T5" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2">
         <v>3</v>
       </c>
       <c r="C6" s="2">
-        <v>3.6727999999999997E-2</v>
+        <v>3.6819999999999999E-2</v>
       </c>
       <c r="D6" s="2">
-        <v>3.6724E-2</v>
+        <v>3.6816000000000002E-2</v>
       </c>
       <c r="E6" s="2">
-        <v>1.9999999999999999E-6</v>
+        <v>3.0000000000000001E-6</v>
       </c>
       <c r="F6" s="2">
         <v>9.9999999999999995E-7</v>
@@ -751,36 +746,36 @@
         <v>0</v>
       </c>
       <c r="H6" s="2">
-        <v>96.162800000000004</v>
+        <v>96.160600000000002</v>
       </c>
       <c r="I6" s="2">
-        <v>96.4923</v>
+        <v>96.476299999999995</v>
       </c>
       <c r="J6" s="2">
-        <v>0.99870000000000003</v>
+        <v>0.99750000000000005</v>
       </c>
       <c r="K6" s="2">
-        <v>0.97350000000000003</v>
-      </c>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" t="s">
+        <v>0.97799999999999998</v>
+      </c>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="T6" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="T6" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
         <v>4</v>
       </c>
       <c r="C7" s="2">
-        <v>3.5619999999999999E-2</v>
+        <v>3.5583999999999998E-2</v>
       </c>
       <c r="D7" s="2">
-        <v>3.5619999999999999E-2</v>
+        <v>3.5583999999999998E-2</v>
       </c>
       <c r="E7" s="2">
         <v>0</v>
@@ -791,40 +786,40 @@
       <c r="G7" s="2">
         <v>0</v>
       </c>
-      <c r="H7" s="3"/>
+      <c r="H7" s="2"/>
       <c r="I7" s="2">
-        <v>96.438000000000002</v>
-      </c>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
+        <v>96.441599999999994</v>
+      </c>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
       <c r="L7" s="2">
         <v>1</v>
       </c>
       <c r="M7" s="2">
-        <v>0.99419999999999997</v>
+        <v>0.99550000000000005</v>
       </c>
       <c r="N7" s="2">
         <v>1</v>
       </c>
-      <c r="O7" t="s">
+      <c r="O7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="T7" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="T7" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
         <v>5</v>
       </c>
       <c r="C8" s="2">
-        <v>3.8384000000000001E-2</v>
+        <v>3.8261000000000003E-2</v>
       </c>
       <c r="D8" s="2">
-        <v>3.8379999999999997E-2</v>
+        <v>3.8255999999999998E-2</v>
       </c>
       <c r="E8" s="2">
-        <v>3.9999999999999998E-6</v>
+        <v>5.0000000000000004E-6</v>
       </c>
       <c r="F8" s="2">
         <v>0</v>
@@ -833,36 +828,36 @@
         <v>0</v>
       </c>
       <c r="H8" s="2">
-        <v>96.170500000000004</v>
+        <v>96.187899999999999</v>
       </c>
       <c r="I8" s="2">
-        <v>96.153400000000005</v>
+        <v>96.160899999999998</v>
       </c>
       <c r="J8" s="2">
-        <v>0.99890000000000001</v>
+        <v>0.99819999999999998</v>
       </c>
       <c r="K8" s="2">
         <v>0.99960000000000004</v>
       </c>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" t="s">
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="T8" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="T8" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2">
         <v>6</v>
       </c>
       <c r="C9" s="2">
-        <v>3.6997000000000002E-2</v>
+        <v>3.6760000000000001E-2</v>
       </c>
       <c r="D9" s="2">
-        <v>3.6996000000000001E-2</v>
+        <v>3.6759E-2</v>
       </c>
       <c r="E9" s="2">
         <v>9.9999999999999995E-7</v>
@@ -874,45 +869,45 @@
         <v>0</v>
       </c>
       <c r="H9" s="2">
-        <v>96.127499999999998</v>
+        <v>96.128399999999999</v>
       </c>
       <c r="I9" s="2">
-        <v>96.408299999999997</v>
+        <v>96.448599999999999</v>
       </c>
       <c r="J9" s="2">
-        <v>0.99670000000000003</v>
+        <v>0.99770000000000003</v>
       </c>
       <c r="K9" s="2">
-        <v>0.98299999999999998</v>
-      </c>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" t="s">
+        <v>0.9879</v>
+      </c>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="Q9">
-        <v>96.365499999999997</v>
-      </c>
-      <c r="R9">
-        <v>0.98309999999999997</v>
-      </c>
-      <c r="T9" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="Q9" s="3">
+        <v>96.395200000000003</v>
+      </c>
+      <c r="R9" s="3">
+        <v>0.98080000000000001</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
         <v>7</v>
       </c>
       <c r="C10" s="2">
-        <v>16579.468714999999</v>
+        <v>16177.468803</v>
       </c>
       <c r="D10" s="2">
-        <v>16579.468670999999</v>
+        <v>16177.468709000001</v>
       </c>
       <c r="E10" s="2">
-        <v>4.3999999999999999E-5</v>
+        <v>9.3999999999999994E-5</v>
       </c>
       <c r="F10" s="2">
         <v>0</v>
@@ -921,36 +916,36 @@
         <v>0</v>
       </c>
       <c r="H10" s="2">
-        <v>89.872200000000007</v>
+        <v>89.008300000000006</v>
       </c>
       <c r="I10" s="2">
-        <v>87.011499999999998</v>
+        <v>87.822400000000002</v>
       </c>
       <c r="J10" s="2">
-        <v>0.99450000000000005</v>
+        <v>0.99429999999999996</v>
       </c>
       <c r="K10" s="2">
-        <v>0.95040000000000002</v>
-      </c>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" t="s">
+        <v>0.95250000000000001</v>
+      </c>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
+      <c r="O10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="T10" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="T10" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B11" s="2">
         <v>8</v>
       </c>
       <c r="C11" s="2">
-        <v>3.5661999999999999E-2</v>
+        <v>3.5630000000000002E-2</v>
       </c>
       <c r="D11" s="2">
-        <v>3.5660999999999998E-2</v>
+        <v>3.5630000000000002E-2</v>
       </c>
       <c r="E11" s="2">
         <v>0</v>
@@ -962,83 +957,80 @@
         <v>0</v>
       </c>
       <c r="H11" s="2">
-        <v>96.433899999999994</v>
-      </c>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
+        <v>96.436999999999998</v>
+      </c>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
       <c r="L11" s="2">
-        <v>0.999</v>
+        <v>0.99880000000000002</v>
       </c>
       <c r="M11" s="2">
-        <v>0.98580000000000001</v>
+        <v>0.98089999999999999</v>
       </c>
       <c r="N11" s="2">
-        <v>0.99950000000000006</v>
-      </c>
-      <c r="O11" t="s">
+        <v>0.99919999999999998</v>
+      </c>
+      <c r="O11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="T11" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="T11" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B12" s="2">
         <v>9</v>
       </c>
       <c r="C12" s="2">
-        <v>4.4505000000000003E-2</v>
+        <v>5.1501999999999999E-2</v>
       </c>
       <c r="D12" s="2">
-        <v>4.2646999999999997E-2</v>
+        <v>5.1501999999999999E-2</v>
       </c>
       <c r="E12" s="2">
         <v>0</v>
       </c>
       <c r="F12" s="2">
-        <v>1.503E-3</v>
+        <v>0</v>
       </c>
       <c r="G12" s="2">
-        <v>3.5500000000000001E-4</v>
-      </c>
-      <c r="H12" s="3"/>
+        <v>0</v>
+      </c>
+      <c r="H12" s="2"/>
       <c r="I12" s="2">
-        <v>95.735299999999995</v>
-      </c>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
+        <v>94.849800000000002</v>
+      </c>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
       <c r="L12" s="2">
-        <v>0.99980000000000002</v>
+        <v>0.99680000000000002</v>
       </c>
       <c r="M12" s="2">
-        <v>0.98170000000000002</v>
+        <v>0.96850000000000003</v>
       </c>
       <c r="N12" s="2">
-        <v>0.99970000000000003</v>
-      </c>
-      <c r="O12" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>19</v>
+        <v>0.99829999999999997</v>
+      </c>
+      <c r="O12" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="U12" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="2:21" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="U12" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B13" s="2">
         <v>10</v>
       </c>
       <c r="C13" s="2">
-        <v>0.38922499999999999</v>
+        <v>0.38962000000000002</v>
       </c>
       <c r="D13" s="2">
-        <v>0.38922400000000001</v>
+        <v>0.38962000000000002</v>
       </c>
       <c r="E13" s="2">
         <v>0</v>
@@ -1050,27 +1042,27 @@
         <v>0</v>
       </c>
       <c r="H13" s="2">
-        <v>61.058300000000003</v>
-      </c>
-      <c r="I13" s="3"/>
+        <v>61.042999999999999</v>
+      </c>
+      <c r="I13" s="2"/>
       <c r="J13" s="2">
-        <v>0.99939999999999996</v>
-      </c>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-      <c r="O13" t="s">
+        <v>0.99919999999999998</v>
+      </c>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="3" t="s">
         <v>14</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="U13" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14" spans="2:21" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="U13" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2">
         <v>11</v>
       </c>
@@ -1089,12 +1081,10 @@
       <c r="G14" s="2">
         <v>0</v>
       </c>
-      <c r="H14" s="3"/>
+      <c r="H14" s="2"/>
       <c r="I14" s="2">
         <v>20.811399999999999</v>
       </c>
-      <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
       <c r="L14" s="2">
         <v>0.99719999999999998</v>
       </c>
@@ -1104,87 +1094,87 @@
       <c r="N14" s="2">
         <v>0.99639999999999995</v>
       </c>
-      <c r="O14" t="s">
+      <c r="O14" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="T14" s="4" t="s">
-        <v>22</v>
+      <c r="T14" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
     </row>
     <row r="16" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
-      <c r="N19" s="2"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
Stable equality unit tests added
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\CMTF_AOADMM_refactor\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6181D77E-22A0-42A5-9702-15DF7ED9DC6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB3C0E9-EBA1-467C-9A54-BA49F251CBF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
@@ -138,7 +138,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -157,6 +157,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -170,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -183,6 +189,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -591,48 +601,48 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="2">
+    <row r="3" spans="2:21" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="6">
         <v>1</v>
       </c>
-      <c r="C3" s="2">
-        <v>0</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2">
-        <v>0</v>
-      </c>
-      <c r="F3" s="2">
-        <v>0</v>
-      </c>
-      <c r="G3" s="2">
-        <v>0</v>
-      </c>
-      <c r="H3" s="2">
+      <c r="C3" s="6">
+        <v>0</v>
+      </c>
+      <c r="D3" s="6">
+        <v>0</v>
+      </c>
+      <c r="E3" s="6">
+        <v>0</v>
+      </c>
+      <c r="F3" s="6">
+        <v>0</v>
+      </c>
+      <c r="G3" s="6">
+        <v>0</v>
+      </c>
+      <c r="H3" s="6">
         <v>100</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="6">
         <v>100</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="6">
         <v>1</v>
       </c>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2">
+      <c r="K3" s="6"/>
+      <c r="L3" s="6">
         <v>1</v>
       </c>
-      <c r="M3" s="2">
+      <c r="M3" s="6">
         <v>0.999</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="6">
         <v>1</v>
       </c>
-      <c r="O3" s="3" t="s">
+      <c r="O3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="T3" s="2" t="s">
+      <c r="T3" s="6" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Modify flaky test for script 4 for macOS
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\CMTF_AOADMM_refactor\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB3C0E9-EBA1-467C-9A54-BA49F251CBF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BACB4B41-4F48-404C-B23A-9697B48DFB73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="25">
   <si>
     <t>Example script number</t>
   </si>
@@ -101,22 +101,16 @@
     <t>Correct</t>
   </si>
   <si>
-    <t>Refactor</t>
-  </si>
-  <si>
-    <t>Broken</t>
-  </si>
-  <si>
-    <t>Correct?</t>
-  </si>
-  <si>
-    <t>Fig different?</t>
-  </si>
-  <si>
     <t>0,000007</t>
   </si>
   <si>
     <t>Run under rng(123, 'twister')</t>
+  </si>
+  <si>
+    <t>Figures</t>
+  </si>
+  <si>
+    <t>Incorrect</t>
   </si>
 </sst>
 </file>
@@ -138,7 +132,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -163,6 +157,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -176,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -193,6 +199,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -527,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6001F213-F06F-43A9-9C65-6A6D4326F486}">
-  <dimension ref="B1:U19"/>
+  <dimension ref="B1:T19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
@@ -543,12 +555,12 @@
     <col min="20" max="20" width="15.140625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="2:21" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="2:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
@@ -597,11 +609,11 @@
       <c r="R2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="T2" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="2:21" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T2" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="6">
         <v>1</v>
       </c>
@@ -646,7 +658,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
@@ -657,7 +669,7 @@
         <v>0.22126100000000001</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F4" s="2">
         <v>3.6000000000000001E-5</v>
@@ -665,10 +677,10 @@
       <c r="G4" s="2">
         <v>2.395E-3</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="8">
         <v>80.028000000000006</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="8">
         <v>79.271799999999999</v>
       </c>
       <c r="J4" s="2">
@@ -678,10 +690,10 @@
       <c r="L4" s="2">
         <v>0.99870000000000003</v>
       </c>
-      <c r="M4" s="2">
+      <c r="M4" s="8">
         <v>0.94030000000000002</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="8">
         <v>0.99660000000000004</v>
       </c>
       <c r="O4" s="3" t="s">
@@ -691,222 +703,222 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="2">
+    <row r="5" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="6">
         <v>2</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="6">
         <v>0.18159600000000001</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="6">
         <v>0.18159500000000001</v>
       </c>
-      <c r="E5" s="2">
-        <v>0</v>
-      </c>
-      <c r="F5" s="2">
-        <v>0</v>
-      </c>
-      <c r="G5" s="2">
-        <v>0</v>
-      </c>
-      <c r="H5" s="2">
+      <c r="E5" s="6">
+        <v>0</v>
+      </c>
+      <c r="F5" s="6">
+        <v>0</v>
+      </c>
+      <c r="G5" s="6">
+        <v>0</v>
+      </c>
+      <c r="H5" s="6">
         <v>82.649000000000001</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="6">
         <v>81.117699999999999</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="6">
         <v>0.91859999999999997</v>
       </c>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2">
+      <c r="K5" s="6"/>
+      <c r="L5" s="6">
         <v>0.97509999999999997</v>
       </c>
-      <c r="M5" s="2">
+      <c r="M5" s="6">
         <v>0.93130000000000002</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="6">
         <v>0.9909</v>
       </c>
-      <c r="O5" s="3" t="s">
+      <c r="O5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="T5" s="2" t="s">
+      <c r="T5" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="2">
+    <row r="6" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="6">
         <v>3</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="6">
         <v>3.6819999999999999E-2</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="6">
         <v>3.6816000000000002E-2</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="6">
         <v>3.0000000000000001E-6</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="6">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="G6" s="2">
-        <v>0</v>
-      </c>
-      <c r="H6" s="2">
+      <c r="G6" s="6">
+        <v>0</v>
+      </c>
+      <c r="H6" s="6">
         <v>96.160600000000002</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="6">
         <v>96.476299999999995</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="6">
         <v>0.99750000000000005</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="6">
         <v>0.97799999999999998</v>
       </c>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="3" t="s">
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="T6" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="2">
+      <c r="T6" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="6">
         <v>4</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="6">
         <v>3.5583999999999998E-2</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="6">
         <v>3.5583999999999998E-2</v>
       </c>
-      <c r="E7" s="2">
-        <v>0</v>
-      </c>
-      <c r="F7" s="2">
-        <v>0</v>
-      </c>
-      <c r="G7" s="2">
-        <v>0</v>
-      </c>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2">
+      <c r="E7" s="6">
+        <v>0</v>
+      </c>
+      <c r="F7" s="6">
+        <v>0</v>
+      </c>
+      <c r="G7" s="6">
+        <v>0</v>
+      </c>
+      <c r="H7" s="6"/>
+      <c r="I7" s="9">
         <v>96.441599999999994</v>
       </c>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2">
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6">
         <v>1</v>
       </c>
-      <c r="M7" s="2">
+      <c r="M7" s="6">
         <v>0.99550000000000005</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="6">
         <v>1</v>
       </c>
-      <c r="O7" s="3" t="s">
+      <c r="O7" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="T7" s="2" t="s">
+      <c r="T7" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="2">
+    <row r="8" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="6">
         <v>5</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="6">
         <v>3.8261000000000003E-2</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="6">
         <v>3.8255999999999998E-2</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="6">
         <v>5.0000000000000004E-6</v>
       </c>
-      <c r="F8" s="2">
-        <v>0</v>
-      </c>
-      <c r="G8" s="2">
-        <v>0</v>
-      </c>
-      <c r="H8" s="2">
+      <c r="F8" s="6">
+        <v>0</v>
+      </c>
+      <c r="G8" s="6">
+        <v>0</v>
+      </c>
+      <c r="H8" s="6">
         <v>96.187899999999999</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="6">
         <v>96.160899999999998</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="6">
         <v>0.99819999999999998</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="6">
         <v>0.99960000000000004</v>
       </c>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="3" t="s">
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="6"/>
+      <c r="O8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="T8" s="2" t="s">
+      <c r="T8" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="2">
+    <row r="9" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="6">
         <v>6</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="6">
         <v>3.6760000000000001E-2</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="6">
         <v>3.6759E-2</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="6">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="F9" s="2">
-        <v>0</v>
-      </c>
-      <c r="G9" s="2">
-        <v>0</v>
-      </c>
-      <c r="H9" s="2">
+      <c r="F9" s="6">
+        <v>0</v>
+      </c>
+      <c r="G9" s="6">
+        <v>0</v>
+      </c>
+      <c r="H9" s="6">
         <v>96.128399999999999</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="6">
         <v>96.448599999999999</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="6">
         <v>0.99770000000000003</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="6">
         <v>0.9879</v>
       </c>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
-      <c r="O9" s="3" t="s">
+      <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
+      <c r="N9" s="6"/>
+      <c r="O9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="Q9" s="3">
+      <c r="Q9" s="7">
         <v>96.395200000000003</v>
       </c>
-      <c r="R9" s="3">
+      <c r="R9" s="7">
         <v>0.98080000000000001</v>
       </c>
-      <c r="T9" s="2" t="s">
+      <c r="T9" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
         <v>7</v>
       </c>
@@ -925,10 +937,10 @@
       <c r="G10" s="2">
         <v>0</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="8">
         <v>89.008300000000006</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="8">
         <v>87.822400000000002</v>
       </c>
       <c r="J10" s="2">
@@ -943,11 +955,11 @@
       <c r="O10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="T10" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T10" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="2:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B11" s="2">
         <v>8</v>
       </c>
@@ -966,152 +978,146 @@
       <c r="G11" s="2">
         <v>0</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="8">
         <v>96.436999999999998</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
-      <c r="L11" s="2">
+      <c r="L11" s="8">
         <v>0.99880000000000002</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="8">
         <v>0.98089999999999999</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="8">
         <v>0.99919999999999998</v>
       </c>
       <c r="O11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="T11" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="2">
+      <c r="T11" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="6">
         <v>9</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="6">
         <v>5.1501999999999999E-2</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="6">
         <v>5.1501999999999999E-2</v>
       </c>
-      <c r="E12" s="2">
-        <v>0</v>
-      </c>
-      <c r="F12" s="2">
-        <v>0</v>
-      </c>
-      <c r="G12" s="2">
-        <v>0</v>
-      </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2">
+      <c r="E12" s="6">
+        <v>0</v>
+      </c>
+      <c r="F12" s="6">
+        <v>0</v>
+      </c>
+      <c r="G12" s="6">
+        <v>0</v>
+      </c>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6">
         <v>94.849800000000002</v>
       </c>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2">
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6">
         <v>0.99680000000000002</v>
       </c>
-      <c r="M12" s="2">
+      <c r="M12" s="6">
         <v>0.96850000000000003</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="6">
         <v>0.99829999999999997</v>
       </c>
-      <c r="O12" s="3" t="s">
+      <c r="O12" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="T12" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="U12" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="2">
+      <c r="T12" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="6">
         <v>10</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="6">
         <v>0.38962000000000002</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="6">
         <v>0.38962000000000002</v>
       </c>
-      <c r="E13" s="2">
-        <v>0</v>
-      </c>
-      <c r="F13" s="2">
-        <v>0</v>
-      </c>
-      <c r="G13" s="2">
-        <v>0</v>
-      </c>
-      <c r="H13" s="2">
+      <c r="E13" s="6">
+        <v>0</v>
+      </c>
+      <c r="F13" s="6">
+        <v>0</v>
+      </c>
+      <c r="G13" s="6">
+        <v>0</v>
+      </c>
+      <c r="H13" s="6">
         <v>61.042999999999999</v>
       </c>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2">
+      <c r="I13" s="6"/>
+      <c r="J13" s="6">
         <v>0.99919999999999998</v>
       </c>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="3" t="s">
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="T13" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="U13" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="2:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="2">
+      <c r="T13" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="6">
         <v>11</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="6">
         <v>3820743.9982230002</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="6">
         <v>3820743.9982230002</v>
       </c>
-      <c r="E14" s="2">
-        <v>0</v>
-      </c>
-      <c r="F14" s="2">
-        <v>0</v>
-      </c>
-      <c r="G14" s="2">
-        <v>0</v>
-      </c>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2">
+      <c r="E14" s="6">
+        <v>0</v>
+      </c>
+      <c r="F14" s="6">
+        <v>0</v>
+      </c>
+      <c r="G14" s="6">
+        <v>0</v>
+      </c>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6">
         <v>20.811399999999999</v>
       </c>
-      <c r="L14" s="2">
+      <c r="L14" s="6">
         <v>0.99719999999999998</v>
       </c>
-      <c r="M14" s="2">
+      <c r="M14" s="6">
         <v>0.97660000000000002</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="6">
         <v>0.99639999999999995</v>
       </c>
-      <c r="O14" s="3" t="s">
+      <c r="O14" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="T14" s="2" t="s">
+      <c r="T14" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -1126,7 +1132,7 @@
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
     </row>
-    <row r="16" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>

</xml_diff>

<commit_message>
Changed random seed for script 1a
This way it converges
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\CMTF_AOADMM_refactor\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BACB4B41-4F48-404C-B23A-9697B48DFB73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB165C2A-6B05-4CEB-8B8C-997235AFB662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="25">
   <si>
     <t>Example script number</t>
   </si>
@@ -95,22 +95,22 @@
     <t>FMS3</t>
   </si>
   <si>
-    <t>maxIterations</t>
-  </si>
-  <si>
     <t>Correct</t>
   </si>
   <si>
-    <t>0,000007</t>
-  </si>
-  <si>
-    <t>Run under rng(123, 'twister')</t>
-  </si>
-  <si>
     <t>Figures</t>
   </si>
   <si>
     <t>Incorrect</t>
+  </si>
+  <si>
+    <t>RNG</t>
+  </si>
+  <si>
+    <t>rng(123, 'twister')</t>
+  </si>
+  <si>
+    <t>rng(234, 'twister')</t>
   </si>
 </sst>
 </file>
@@ -539,9 +539,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6001F213-F06F-43A9-9C65-6A6D4326F486}">
-  <dimension ref="B1:T19"/>
+  <dimension ref="A2:T19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
@@ -555,12 +556,10 @@
     <col min="20" max="20" width="15.140625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
+    <row r="2" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="2:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
@@ -610,10 +609,13 @@
         <v>18</v>
       </c>
       <c r="T2" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="3" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="6">
         <v>1</v>
       </c>
@@ -655,55 +657,59 @@
         <v>15</v>
       </c>
       <c r="T3" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="2:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="2">
-        <v>0.22369900000000001</v>
+        <v>0.220301</v>
       </c>
       <c r="D4" s="2">
-        <v>0.22126100000000001</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>21</v>
+        <v>0.220301</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0</v>
       </c>
       <c r="F4" s="2">
-        <v>3.6000000000000001E-5</v>
+        <v>0</v>
       </c>
       <c r="G4" s="2">
-        <v>2.395E-3</v>
+        <v>0</v>
       </c>
       <c r="H4" s="8">
-        <v>80.028000000000006</v>
+        <v>80.003900000000002</v>
       </c>
       <c r="I4" s="8">
-        <v>79.271799999999999</v>
+        <v>79.471299999999999</v>
       </c>
       <c r="J4" s="2">
-        <v>0.99760000000000004</v>
+        <v>0.998</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2">
-        <v>0.99870000000000003</v>
+        <v>0.99909999999999999</v>
       </c>
       <c r="M4" s="8">
-        <v>0.94030000000000002</v>
+        <v>0.9667</v>
       </c>
       <c r="N4" s="8">
-        <v>0.99660000000000004</v>
+        <v>0.99909999999999999</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="T4" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+      <c r="T4" s="2"/>
+    </row>
+    <row r="5" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="B5" s="6">
         <v>2</v>
       </c>
@@ -745,10 +751,13 @@
         <v>14</v>
       </c>
       <c r="T5" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="B6" s="6">
         <v>3</v>
       </c>
@@ -786,10 +795,13 @@
         <v>14</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="B7" s="6">
         <v>4</v>
       </c>
@@ -827,10 +839,13 @@
         <v>14</v>
       </c>
       <c r="T7" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="B8" s="6">
         <v>5</v>
       </c>
@@ -868,10 +883,13 @@
         <v>14</v>
       </c>
       <c r="T8" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="B9" s="6">
         <v>6</v>
       </c>
@@ -915,10 +933,13 @@
         <v>0.98080000000000001</v>
       </c>
       <c r="T9" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="2:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="B10" s="2">
         <v>7</v>
       </c>
@@ -956,10 +977,13 @@
         <v>14</v>
       </c>
       <c r="T10" s="8" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="2:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="B11" s="2">
         <v>8</v>
       </c>
@@ -997,10 +1021,13 @@
         <v>14</v>
       </c>
       <c r="T11" s="8" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="B12" s="6">
         <v>9</v>
       </c>
@@ -1038,10 +1065,13 @@
         <v>14</v>
       </c>
       <c r="T12" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="B13" s="6">
         <v>10</v>
       </c>
@@ -1075,10 +1105,13 @@
         <v>14</v>
       </c>
       <c r="T13" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="2:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="B14" s="6">
         <v>11</v>
       </c>
@@ -1114,10 +1147,10 @@
         <v>14</v>
       </c>
       <c r="T14" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="2:20" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -1132,7 +1165,7 @@
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
     </row>
-    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>

</xml_diff>

<commit_message>
Internal case structure fix
G was not given back by ADMM_constrained_only in some cases
This should fix the tests
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\CMTF_AOADMM_refactor\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB165C2A-6B05-4CEB-8B8C-997235AFB662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E23ABCC-DAD3-4080-A00D-3804C54141EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
@@ -1021,7 +1021,7 @@
         <v>14</v>
       </c>
       <c r="T11" s="8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Tighten script 1a and 7 tests again
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\CMTF_AOADMM_refactor\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E23ABCC-DAD3-4080-A00D-3804C54141EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9A5792D-7247-41E6-A45C-6F02CCBBCB2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
@@ -980,47 +980,47 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="6">
         <v>8</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="6">
         <v>3.5630000000000002E-2</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="6">
         <v>3.5630000000000002E-2</v>
       </c>
-      <c r="E11" s="2">
-        <v>0</v>
-      </c>
-      <c r="F11" s="2">
-        <v>0</v>
-      </c>
-      <c r="G11" s="2">
-        <v>0</v>
-      </c>
-      <c r="H11" s="8">
+      <c r="E11" s="6">
+        <v>0</v>
+      </c>
+      <c r="F11" s="6">
+        <v>0</v>
+      </c>
+      <c r="G11" s="6">
+        <v>0</v>
+      </c>
+      <c r="H11" s="6">
         <v>96.436999999999998</v>
       </c>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="8">
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="6">
         <v>0.99880000000000002</v>
       </c>
-      <c r="M11" s="8">
+      <c r="M11" s="6">
         <v>0.98089999999999999</v>
       </c>
-      <c r="N11" s="8">
+      <c r="N11" s="6">
         <v>0.99919999999999998</v>
       </c>
-      <c r="O11" s="3" t="s">
+      <c r="O11" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="T11" s="8" t="s">
+      <c r="T11" s="6" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add diagnostics to script 1a test
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\CMTF_AOADMM_refactor\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9A5792D-7247-41E6-A45C-6F02CCBBCB2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2236ED06-4F19-4F13-AD3C-68C6CFAACD47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="24">
   <si>
     <t>Example script number</t>
   </si>
@@ -99,9 +99,6 @@
   </si>
   <si>
     <t>Figures</t>
-  </si>
-  <si>
-    <t>Incorrect</t>
   </si>
   <si>
     <t>RNG</t>
@@ -558,7 +555,7 @@
   <sheetData>
     <row r="2" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>0</v>
@@ -614,7 +611,7 @@
     </row>
     <row r="3" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" s="6">
         <v>1</v>
@@ -662,7 +659,7 @@
     </row>
     <row r="4" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>13</v>
@@ -708,7 +705,7 @@
     </row>
     <row r="5" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5" s="6">
         <v>2</v>
@@ -756,7 +753,7 @@
     </row>
     <row r="6" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B6" s="6">
         <v>3</v>
@@ -800,7 +797,7 @@
     </row>
     <row r="7" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7" s="6">
         <v>4</v>
@@ -844,7 +841,7 @@
     </row>
     <row r="8" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B8" s="6">
         <v>5</v>
@@ -888,7 +885,7 @@
     </row>
     <row r="9" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" s="6">
         <v>6</v>
@@ -936,53 +933,53 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="2">
+    <row r="10" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="6">
         <v>7</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="6">
         <v>16177.468803</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="6">
         <v>16177.468709000001</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="6">
         <v>9.3999999999999994E-5</v>
       </c>
-      <c r="F10" s="2">
-        <v>0</v>
-      </c>
-      <c r="G10" s="2">
-        <v>0</v>
-      </c>
-      <c r="H10" s="8">
+      <c r="F10" s="6">
+        <v>0</v>
+      </c>
+      <c r="G10" s="6">
+        <v>0</v>
+      </c>
+      <c r="H10" s="6">
         <v>89.008300000000006</v>
       </c>
-      <c r="I10" s="8">
+      <c r="I10" s="6">
         <v>87.822400000000002</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="6">
         <v>0.99429999999999996</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="6">
         <v>0.95250000000000001</v>
       </c>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
-      <c r="O10" s="3" t="s">
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="T10" s="8" t="s">
-        <v>21</v>
+      <c r="T10" s="6" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B11" s="6">
         <v>8</v>
@@ -1026,7 +1023,7 @@
     </row>
     <row r="12" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B12" s="6">
         <v>9</v>
@@ -1070,7 +1067,7 @@
     </row>
     <row r="13" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" s="6">
         <v>10</v>
@@ -1110,7 +1107,7 @@
     </row>
     <row r="14" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B14" s="6">
         <v>11</v>

</xml_diff>

<commit_message>
Added outerIters to tests
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\CMTF_AOADMM_refactor\examples\ExpectedOutput\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\Refactor_experiment\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2236ED06-4F19-4F13-AD3C-68C6CFAACD47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B74A09C-F2D2-4EA3-8CF7-1379F41D62A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="25">
   <si>
     <t>Example script number</t>
   </si>
@@ -108,6 +108,9 @@
   </si>
   <si>
     <t>rng(234, 'twister')</t>
+  </si>
+  <si>
+    <t>OuterIters</t>
   </si>
 </sst>
 </file>
@@ -605,6 +608,9 @@
       <c r="R2" s="4" t="s">
         <v>18</v>
       </c>
+      <c r="S2" s="5" t="s">
+        <v>24</v>
+      </c>
       <c r="T2" s="5" t="s">
         <v>20</v>
       </c>
@@ -653,6 +659,9 @@
       <c r="O3" s="7" t="s">
         <v>15</v>
       </c>
+      <c r="S3" s="7">
+        <v>398</v>
+      </c>
       <c r="T3" s="6" t="s">
         <v>19</v>
       </c>
@@ -701,6 +710,9 @@
       <c r="O4" s="3" t="s">
         <v>14</v>
       </c>
+      <c r="S4" s="3">
+        <v>75</v>
+      </c>
       <c r="T4" s="2"/>
     </row>
     <row r="5" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -746,6 +758,9 @@
       </c>
       <c r="O5" s="7" t="s">
         <v>14</v>
+      </c>
+      <c r="S5" s="7">
+        <v>246</v>
       </c>
       <c r="T5" s="6" t="s">
         <v>19</v>
@@ -791,6 +806,9 @@
       <c r="O6" s="7" t="s">
         <v>14</v>
       </c>
+      <c r="S6" s="7">
+        <v>125</v>
+      </c>
       <c r="T6" s="6" t="s">
         <v>19</v>
       </c>
@@ -834,6 +852,9 @@
       </c>
       <c r="O7" s="7" t="s">
         <v>14</v>
+      </c>
+      <c r="S7" s="7">
+        <v>182</v>
       </c>
       <c r="T7" s="6" t="s">
         <v>19</v>
@@ -879,6 +900,9 @@
       <c r="O8" s="7" t="s">
         <v>14</v>
       </c>
+      <c r="S8" s="7">
+        <v>15</v>
+      </c>
       <c r="T8" s="6" t="s">
         <v>19</v>
       </c>
@@ -929,6 +953,9 @@
       <c r="R9" s="7">
         <v>0.98080000000000001</v>
       </c>
+      <c r="S9" s="7">
+        <v>126</v>
+      </c>
       <c r="T9" s="6" t="s">
         <v>19</v>
       </c>
@@ -973,6 +1000,9 @@
       <c r="O10" s="7" t="s">
         <v>14</v>
       </c>
+      <c r="S10" s="7">
+        <v>32</v>
+      </c>
       <c r="T10" s="6" t="s">
         <v>19</v>
       </c>
@@ -1017,6 +1047,9 @@
       <c r="O11" s="7" t="s">
         <v>14</v>
       </c>
+      <c r="S11" s="7">
+        <v>131</v>
+      </c>
       <c r="T11" s="6" t="s">
         <v>19</v>
       </c>
@@ -1060,6 +1093,9 @@
       </c>
       <c r="O12" s="7" t="s">
         <v>14</v>
+      </c>
+      <c r="S12" s="7">
+        <v>190</v>
       </c>
       <c r="T12" s="6" t="s">
         <v>19</v>
@@ -1101,6 +1137,9 @@
       <c r="O13" s="7" t="s">
         <v>14</v>
       </c>
+      <c r="S13" s="7">
+        <v>805</v>
+      </c>
       <c r="T13" s="6" t="s">
         <v>19</v>
       </c>
@@ -1142,6 +1181,9 @@
       </c>
       <c r="O14" s="7" t="s">
         <v>14</v>
+      </c>
+      <c r="S14" s="7">
+        <v>1862</v>
       </c>
       <c r="T14" s="6" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Reproducibility fix to create_data smooth bks
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\Refactor_experiment\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B74A09C-F2D2-4EA3-8CF7-1379F41D62A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E528303C-E546-4941-9140-FA09577B42EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
@@ -674,10 +674,10 @@
         <v>13</v>
       </c>
       <c r="C4" s="2">
-        <v>0.220301</v>
+        <v>0.221914</v>
       </c>
       <c r="D4" s="2">
-        <v>0.220301</v>
+        <v>0.221913</v>
       </c>
       <c r="E4" s="2">
         <v>0</v>
@@ -689,29 +689,29 @@
         <v>0</v>
       </c>
       <c r="H4" s="8">
-        <v>80.003900000000002</v>
+        <v>79.987399999999994</v>
       </c>
       <c r="I4" s="8">
-        <v>79.471299999999999</v>
+        <v>79.3005</v>
       </c>
       <c r="J4" s="2">
-        <v>0.998</v>
+        <v>0.99790000000000001</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2">
-        <v>0.99909999999999999</v>
+        <v>0.99890000000000001</v>
       </c>
       <c r="M4" s="8">
-        <v>0.9667</v>
+        <v>0.9607</v>
       </c>
       <c r="N4" s="8">
-        <v>0.99909999999999999</v>
-      </c>
-      <c r="O4" s="3" t="s">
+        <v>0.999</v>
+      </c>
+      <c r="O4" s="7" t="s">
         <v>14</v>
       </c>
       <c r="S4" s="3">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="T4" s="2"/>
     </row>

</xml_diff>

<commit_message>
svd fix to smooth bks
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\Refactor_experiment\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E528303C-E546-4941-9140-FA09577B42EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8D695BA-5D05-45E6-87CA-4C40390228B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
@@ -674,10 +674,10 @@
         <v>13</v>
       </c>
       <c r="C4" s="2">
-        <v>0.221914</v>
+        <v>0.221163</v>
       </c>
       <c r="D4" s="2">
-        <v>0.221913</v>
+        <v>0.221163</v>
       </c>
       <c r="E4" s="2">
         <v>0</v>
@@ -689,10 +689,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="8">
-        <v>79.987399999999994</v>
+        <v>79.9893</v>
       </c>
       <c r="I4" s="8">
-        <v>79.3005</v>
+        <v>79.453100000000006</v>
       </c>
       <c r="J4" s="2">
         <v>0.99790000000000001</v>
@@ -702,16 +702,16 @@
         <v>0.99890000000000001</v>
       </c>
       <c r="M4" s="8">
-        <v>0.9607</v>
+        <v>0.97419999999999995</v>
       </c>
       <c r="N4" s="8">
-        <v>0.999</v>
+        <v>0.99960000000000004</v>
       </c>
       <c r="O4" s="7" t="s">
         <v>14</v>
       </c>
       <c r="S4" s="3">
-        <v>69</v>
+        <v>115</v>
       </c>
       <c r="T4" s="2"/>
     </row>

</xml_diff>

<commit_message>
Replace svd with qr in smooth bks
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\Refactor_experiment\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8D695BA-5D05-45E6-87CA-4C40390228B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63949FAA-14B4-48CC-831A-BFC7539542CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
@@ -674,10 +674,10 @@
         <v>13</v>
       </c>
       <c r="C4" s="2">
-        <v>0.221163</v>
+        <v>0.22161</v>
       </c>
       <c r="D4" s="2">
-        <v>0.221163</v>
+        <v>0.22161</v>
       </c>
       <c r="E4" s="2">
         <v>0</v>
@@ -692,17 +692,16 @@
         <v>79.9893</v>
       </c>
       <c r="I4" s="8">
-        <v>79.453100000000006</v>
+        <v>79.316299999999998</v>
       </c>
       <c r="J4" s="2">
         <v>0.99790000000000001</v>
       </c>
-      <c r="K4" s="2"/>
       <c r="L4" s="2">
         <v>0.99890000000000001</v>
       </c>
-      <c r="M4" s="8">
-        <v>0.97419999999999995</v>
+      <c r="M4" s="2">
+        <v>0.97729999999999995</v>
       </c>
       <c r="N4" s="8">
         <v>0.99960000000000004</v>
@@ -711,7 +710,7 @@
         <v>14</v>
       </c>
       <c r="S4" s="3">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="T4" s="2"/>
     </row>

</xml_diff>

<commit_message>
test script 1a now fixed
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\Refactor_experiment\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63949FAA-14B4-48CC-831A-BFC7539542CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A45DEA99-2B2F-4C91-81A8-292A768B2B60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="25">
   <si>
     <t>Example script number</t>
   </si>
@@ -132,18 +132,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -159,13 +153,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -182,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -198,11 +192,8 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -556,136 +547,136 @@
     <col min="20" max="20" width="15.140625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="Q2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="R2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="S2" s="5" t="s">
+      <c r="S2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="T2" s="5" t="s">
+      <c r="T2" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="4">
         <v>1</v>
       </c>
-      <c r="C3" s="6">
-        <v>0</v>
-      </c>
-      <c r="D3" s="6">
-        <v>0</v>
-      </c>
-      <c r="E3" s="6">
-        <v>0</v>
-      </c>
-      <c r="F3" s="6">
-        <v>0</v>
-      </c>
-      <c r="G3" s="6">
-        <v>0</v>
-      </c>
-      <c r="H3" s="6">
+      <c r="C3" s="4">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4">
         <v>100</v>
       </c>
-      <c r="I3" s="6">
+      <c r="I3" s="4">
         <v>100</v>
       </c>
-      <c r="J3" s="6">
+      <c r="J3" s="4">
         <v>1</v>
       </c>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6">
+      <c r="K3" s="4"/>
+      <c r="L3" s="4">
         <v>1</v>
       </c>
-      <c r="M3" s="6">
+      <c r="M3" s="4">
         <v>0.999</v>
       </c>
-      <c r="N3" s="6">
+      <c r="N3" s="4">
         <v>1</v>
       </c>
-      <c r="O3" s="7" t="s">
+      <c r="O3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="S3" s="7">
+      <c r="S3" s="5">
         <v>398</v>
       </c>
-      <c r="T3" s="6" t="s">
+      <c r="T3" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="8">
         <v>0.22161</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="8">
         <v>0.22161</v>
       </c>
-      <c r="E4" s="2">
-        <v>0</v>
-      </c>
-      <c r="F4" s="2">
-        <v>0</v>
-      </c>
-      <c r="G4" s="2">
+      <c r="E4" s="8">
+        <v>0</v>
+      </c>
+      <c r="F4" s="8">
+        <v>0</v>
+      </c>
+      <c r="G4" s="8">
         <v>0</v>
       </c>
       <c r="H4" s="8">
@@ -694,13 +685,13 @@
       <c r="I4" s="8">
         <v>79.316299999999998</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="8">
         <v>0.99790000000000001</v>
       </c>
-      <c r="L4" s="2">
+      <c r="L4" s="8">
         <v>0.99890000000000001</v>
       </c>
-      <c r="M4" s="2">
+      <c r="M4" s="8">
         <v>0.97729999999999995</v>
       </c>
       <c r="N4" s="8">
@@ -709,482 +700,484 @@
       <c r="O4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="S4" s="3">
+      <c r="S4" s="7">
         <v>114</v>
       </c>
-      <c r="T4" s="2"/>
-    </row>
-    <row r="5" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="T4" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="4">
         <v>2</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="4">
         <v>0.18159600000000001</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="4">
         <v>0.18159500000000001</v>
       </c>
-      <c r="E5" s="6">
-        <v>0</v>
-      </c>
-      <c r="F5" s="6">
-        <v>0</v>
-      </c>
-      <c r="G5" s="6">
-        <v>0</v>
-      </c>
-      <c r="H5" s="6">
+      <c r="E5" s="4">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
         <v>82.649000000000001</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="4">
         <v>81.117699999999999</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="4">
         <v>0.91859999999999997</v>
       </c>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6">
+      <c r="K5" s="4"/>
+      <c r="L5" s="4">
         <v>0.97509999999999997</v>
       </c>
-      <c r="M5" s="6">
+      <c r="M5" s="4">
         <v>0.93130000000000002</v>
       </c>
-      <c r="N5" s="6">
+      <c r="N5" s="4">
         <v>0.9909</v>
       </c>
-      <c r="O5" s="7" t="s">
+      <c r="O5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="S5" s="7">
+      <c r="S5" s="5">
         <v>246</v>
       </c>
-      <c r="T5" s="6" t="s">
+      <c r="T5" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+    <row r="6" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="4">
         <v>3</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="4">
         <v>3.6819999999999999E-2</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
         <v>3.6816000000000002E-2</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="4">
         <v>3.0000000000000001E-6</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="4">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="G6" s="6">
-        <v>0</v>
-      </c>
-      <c r="H6" s="6">
+      <c r="G6" s="4">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4">
         <v>96.160600000000002</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="4">
         <v>96.476299999999995</v>
       </c>
-      <c r="J6" s="6">
+      <c r="J6" s="4">
         <v>0.99750000000000005</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="4">
         <v>0.97799999999999998</v>
       </c>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="7" t="s">
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="S6" s="7">
+      <c r="S6" s="5">
         <v>125</v>
       </c>
-      <c r="T6" s="6" t="s">
+      <c r="T6" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+    <row r="7" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="4">
         <v>4</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="4">
         <v>3.5583999999999998E-2</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="4">
         <v>3.5583999999999998E-2</v>
       </c>
-      <c r="E7" s="6">
-        <v>0</v>
-      </c>
-      <c r="F7" s="6">
-        <v>0</v>
-      </c>
-      <c r="G7" s="6">
-        <v>0</v>
-      </c>
-      <c r="H7" s="6"/>
-      <c r="I7" s="9">
+      <c r="E7" s="4">
+        <v>0</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4"/>
+      <c r="I7" s="6">
         <v>96.441599999999994</v>
       </c>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6">
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4">
         <v>1</v>
       </c>
-      <c r="M7" s="6">
+      <c r="M7" s="4">
         <v>0.99550000000000005</v>
       </c>
-      <c r="N7" s="6">
+      <c r="N7" s="4">
         <v>1</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="O7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="S7" s="7">
+      <c r="S7" s="5">
         <v>182</v>
       </c>
-      <c r="T7" s="6" t="s">
+      <c r="T7" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+    <row r="8" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="4">
         <v>5</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="4">
         <v>3.8261000000000003E-2</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="4">
         <v>3.8255999999999998E-2</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="4">
         <v>5.0000000000000004E-6</v>
       </c>
-      <c r="F8" s="6">
-        <v>0</v>
-      </c>
-      <c r="G8" s="6">
-        <v>0</v>
-      </c>
-      <c r="H8" s="6">
+      <c r="F8" s="4">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4">
         <v>96.187899999999999</v>
       </c>
-      <c r="I8" s="6">
+      <c r="I8" s="4">
         <v>96.160899999999998</v>
       </c>
-      <c r="J8" s="6">
+      <c r="J8" s="4">
         <v>0.99819999999999998</v>
       </c>
-      <c r="K8" s="6">
+      <c r="K8" s="4">
         <v>0.99960000000000004</v>
       </c>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="7" t="s">
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="S8" s="7">
+      <c r="S8" s="5">
         <v>15</v>
       </c>
-      <c r="T8" s="6" t="s">
+      <c r="T8" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+    <row r="9" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="4">
         <v>6</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="4">
         <v>3.6760000000000001E-2</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="4">
         <v>3.6759E-2</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="4">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="F9" s="6">
-        <v>0</v>
-      </c>
-      <c r="G9" s="6">
-        <v>0</v>
-      </c>
-      <c r="H9" s="6">
+      <c r="F9" s="4">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>0</v>
+      </c>
+      <c r="H9" s="4">
         <v>96.128399999999999</v>
       </c>
-      <c r="I9" s="6">
+      <c r="I9" s="4">
         <v>96.448599999999999</v>
       </c>
-      <c r="J9" s="6">
+      <c r="J9" s="4">
         <v>0.99770000000000003</v>
       </c>
-      <c r="K9" s="6">
+      <c r="K9" s="4">
         <v>0.9879</v>
       </c>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="7" t="s">
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="Q9" s="7">
+      <c r="Q9" s="5">
         <v>96.395200000000003</v>
       </c>
-      <c r="R9" s="7">
+      <c r="R9" s="5">
         <v>0.98080000000000001</v>
       </c>
-      <c r="S9" s="7">
+      <c r="S9" s="5">
         <v>126</v>
       </c>
-      <c r="T9" s="6" t="s">
+      <c r="T9" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+    <row r="10" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="6">
+      <c r="B10" s="4">
         <v>7</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="4">
         <v>16177.468803</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="4">
         <v>16177.468709000001</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="4">
         <v>9.3999999999999994E-5</v>
       </c>
-      <c r="F10" s="6">
-        <v>0</v>
-      </c>
-      <c r="G10" s="6">
-        <v>0</v>
-      </c>
-      <c r="H10" s="6">
+      <c r="F10" s="4">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4">
         <v>89.008300000000006</v>
       </c>
-      <c r="I10" s="6">
+      <c r="I10" s="4">
         <v>87.822400000000002</v>
       </c>
-      <c r="J10" s="6">
+      <c r="J10" s="4">
         <v>0.99429999999999996</v>
       </c>
-      <c r="K10" s="6">
+      <c r="K10" s="4">
         <v>0.95250000000000001</v>
       </c>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="7" t="s">
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="S10" s="7">
+      <c r="S10" s="5">
         <v>32</v>
       </c>
-      <c r="T10" s="6" t="s">
+      <c r="T10" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+    <row r="11" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="4">
         <v>8</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="4">
         <v>3.5630000000000002E-2</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="4">
         <v>3.5630000000000002E-2</v>
       </c>
-      <c r="E11" s="6">
-        <v>0</v>
-      </c>
-      <c r="F11" s="6">
-        <v>0</v>
-      </c>
-      <c r="G11" s="6">
-        <v>0</v>
-      </c>
-      <c r="H11" s="6">
+      <c r="E11" s="4">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4">
         <v>96.436999999999998</v>
       </c>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6">
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4">
         <v>0.99880000000000002</v>
       </c>
-      <c r="M11" s="6">
+      <c r="M11" s="4">
         <v>0.98089999999999999</v>
       </c>
-      <c r="N11" s="6">
+      <c r="N11" s="4">
         <v>0.99919999999999998</v>
       </c>
-      <c r="O11" s="7" t="s">
+      <c r="O11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="S11" s="7">
+      <c r="S11" s="5">
         <v>131</v>
       </c>
-      <c r="T11" s="6" t="s">
+      <c r="T11" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+    <row r="12" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="6">
+      <c r="B12" s="4">
         <v>9</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="4">
         <v>5.1501999999999999E-2</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="4">
         <v>5.1501999999999999E-2</v>
       </c>
-      <c r="E12" s="6">
-        <v>0</v>
-      </c>
-      <c r="F12" s="6">
-        <v>0</v>
-      </c>
-      <c r="G12" s="6">
-        <v>0</v>
-      </c>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6">
+      <c r="E12" s="4">
+        <v>0</v>
+      </c>
+      <c r="F12" s="4">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4">
         <v>94.849800000000002</v>
       </c>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6">
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4">
         <v>0.99680000000000002</v>
       </c>
-      <c r="M12" s="6">
+      <c r="M12" s="4">
         <v>0.96850000000000003</v>
       </c>
-      <c r="N12" s="6">
+      <c r="N12" s="4">
         <v>0.99829999999999997</v>
       </c>
-      <c r="O12" s="7" t="s">
+      <c r="O12" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="S12" s="7">
+      <c r="S12" s="5">
         <v>190</v>
       </c>
-      <c r="T12" s="6" t="s">
+      <c r="T12" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
+    <row r="13" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="6">
+      <c r="B13" s="4">
         <v>10</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="4">
         <v>0.38962000000000002</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="4">
         <v>0.38962000000000002</v>
       </c>
-      <c r="E13" s="6">
-        <v>0</v>
-      </c>
-      <c r="F13" s="6">
-        <v>0</v>
-      </c>
-      <c r="G13" s="6">
-        <v>0</v>
-      </c>
-      <c r="H13" s="6">
+      <c r="E13" s="4">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4">
         <v>61.042999999999999</v>
       </c>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6">
+      <c r="I13" s="4"/>
+      <c r="J13" s="4">
         <v>0.99919999999999998</v>
       </c>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="7" t="s">
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="S13" s="7">
+      <c r="S13" s="5">
         <v>805</v>
       </c>
-      <c r="T13" s="6" t="s">
+      <c r="T13" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+    <row r="14" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="6">
+      <c r="B14" s="4">
         <v>11</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="4">
         <v>3820743.9982230002</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="4">
         <v>3820743.9982230002</v>
       </c>
-      <c r="E14" s="6">
-        <v>0</v>
-      </c>
-      <c r="F14" s="6">
-        <v>0</v>
-      </c>
-      <c r="G14" s="6">
-        <v>0</v>
-      </c>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6">
+      <c r="E14" s="4">
+        <v>0</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4">
+        <v>0</v>
+      </c>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4">
         <v>20.811399999999999</v>
       </c>
-      <c r="L14" s="6">
+      <c r="L14" s="4">
         <v>0.99719999999999998</v>
       </c>
-      <c r="M14" s="6">
+      <c r="M14" s="4">
         <v>0.97660000000000002</v>
       </c>
-      <c r="N14" s="6">
+      <c r="N14" s="4">
         <v>0.99639999999999995</v>
       </c>
-      <c r="O14" s="7" t="s">
+      <c r="O14" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="S14" s="7">
+      <c r="S14" s="5">
         <v>1862</v>
       </c>
-      <c r="T14" s="6" t="s">
+      <c r="T14" s="4" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Tightened convergence for test script 7
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\Refactor_experiment\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A45DEA99-2B2F-4C91-81A8-292A768B2B60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3155CBA-A615-46E8-9DDE-C94FF1F84025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="25">
   <si>
     <t>Example script number</t>
   </si>
@@ -132,7 +132,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -163,6 +163,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -176,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -194,6 +200,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -952,52 +962,50 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+    <row r="10" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="10">
         <v>7</v>
       </c>
-      <c r="C10" s="4">
-        <v>16177.468803</v>
-      </c>
-      <c r="D10" s="4">
-        <v>16177.468709000001</v>
-      </c>
-      <c r="E10" s="4">
-        <v>9.3999999999999994E-5</v>
-      </c>
-      <c r="F10" s="4">
-        <v>0</v>
-      </c>
-      <c r="G10" s="4">
-        <v>0</v>
-      </c>
-      <c r="H10" s="4">
-        <v>89.008300000000006</v>
-      </c>
-      <c r="I10" s="4">
-        <v>87.822400000000002</v>
-      </c>
-      <c r="J10" s="4">
-        <v>0.99429999999999996</v>
-      </c>
-      <c r="K10" s="4">
-        <v>0.95250000000000001</v>
-      </c>
-      <c r="L10" s="4"/>
-      <c r="M10" s="4"/>
-      <c r="N10" s="4"/>
+      <c r="C10" s="10">
+        <v>16177.090237</v>
+      </c>
+      <c r="D10" s="10">
+        <v>16177.090227999999</v>
+      </c>
+      <c r="E10" s="10">
+        <v>9.0000000000000002E-6</v>
+      </c>
+      <c r="F10" s="10">
+        <v>0</v>
+      </c>
+      <c r="G10" s="10">
+        <v>0</v>
+      </c>
+      <c r="H10" s="10">
+        <v>89.009299999999996</v>
+      </c>
+      <c r="I10" s="10">
+        <v>87.829099999999997</v>
+      </c>
+      <c r="J10" s="10">
+        <v>0.99419999999999997</v>
+      </c>
+      <c r="K10" s="10">
+        <v>0.9536</v>
+      </c>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
       <c r="O10" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="S10" s="5">
-        <v>32</v>
-      </c>
-      <c r="T10" s="4" t="s">
-        <v>19</v>
-      </c>
+      <c r="S10" s="9">
+        <v>102</v>
+      </c>
+      <c r="T10" s="10"/>
     </row>
     <row r="11" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">

</xml_diff>

<commit_message>
Removed macOS problem for test script 4, updated tests
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\Refactor_experiment\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3155CBA-A615-46E8-9DDE-C94FF1F84025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69B4D063-A29F-4440-B5F9-DB6688916CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -132,7 +132,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -148,12 +148,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -182,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -195,15 +189,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -667,53 +658,53 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="7">
         <v>0.22161</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="7">
         <v>0.22161</v>
       </c>
-      <c r="E4" s="8">
-        <v>0</v>
-      </c>
-      <c r="F4" s="8">
-        <v>0</v>
-      </c>
-      <c r="G4" s="8">
-        <v>0</v>
-      </c>
-      <c r="H4" s="8">
+      <c r="E4" s="7">
+        <v>0</v>
+      </c>
+      <c r="F4" s="7">
+        <v>0</v>
+      </c>
+      <c r="G4" s="7">
+        <v>0</v>
+      </c>
+      <c r="H4" s="7">
         <v>79.9893</v>
       </c>
-      <c r="I4" s="8">
+      <c r="I4" s="7">
         <v>79.316299999999998</v>
       </c>
-      <c r="J4" s="8">
+      <c r="J4" s="7">
         <v>0.99790000000000001</v>
       </c>
-      <c r="L4" s="8">
+      <c r="L4" s="7">
         <v>0.99890000000000001</v>
       </c>
-      <c r="M4" s="8">
+      <c r="M4" s="7">
         <v>0.97729999999999995</v>
       </c>
-      <c r="N4" s="8">
+      <c r="N4" s="7">
         <v>0.99960000000000004</v>
       </c>
-      <c r="O4" s="7" t="s">
+      <c r="O4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="S4" s="7">
+      <c r="S4" s="6">
         <v>114</v>
       </c>
-      <c r="T4" s="8" t="s">
+      <c r="T4" s="7" t="s">
         <v>19</v>
       </c>
     </row>
@@ -815,50 +806,49 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:20" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="9">
         <v>4</v>
       </c>
-      <c r="C7" s="4">
-        <v>3.5583999999999998E-2</v>
-      </c>
-      <c r="D7" s="4">
-        <v>3.5583999999999998E-2</v>
-      </c>
-      <c r="E7" s="4">
-        <v>0</v>
-      </c>
-      <c r="F7" s="4">
-        <v>0</v>
-      </c>
-      <c r="G7" s="4">
-        <v>0</v>
-      </c>
-      <c r="H7" s="4"/>
-      <c r="I7" s="6">
-        <v>96.441599999999994</v>
-      </c>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4">
+      <c r="C7" s="9">
+        <v>3.5564999999999999E-2</v>
+      </c>
+      <c r="D7" s="9">
+        <v>3.5564999999999999E-2</v>
+      </c>
+      <c r="E7" s="9">
+        <v>0</v>
+      </c>
+      <c r="F7" s="9">
+        <v>0</v>
+      </c>
+      <c r="G7" s="9">
+        <v>0</v>
+      </c>
+      <c r="I7" s="9">
+        <v>96.4435</v>
+      </c>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9">
         <v>1</v>
       </c>
-      <c r="M7" s="4">
-        <v>0.99550000000000005</v>
-      </c>
-      <c r="N7" s="4">
+      <c r="M7" s="9">
+        <v>0.99529999999999996</v>
+      </c>
+      <c r="N7" s="9">
         <v>1</v>
       </c>
-      <c r="O7" s="5" t="s">
+      <c r="O7" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="S7" s="5">
-        <v>182</v>
-      </c>
-      <c r="T7" s="4" t="s">
+      <c r="S7" s="8">
+        <v>201</v>
+      </c>
+      <c r="T7" s="9" t="s">
         <v>19</v>
       </c>
     </row>
@@ -962,50 +952,50 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
+    <row r="10" spans="1:20" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="9">
         <v>7</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="9">
         <v>16177.090237</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="9">
         <v>16177.090227999999</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="9">
         <v>9.0000000000000002E-6</v>
       </c>
-      <c r="F10" s="10">
-        <v>0</v>
-      </c>
-      <c r="G10" s="10">
-        <v>0</v>
-      </c>
-      <c r="H10" s="10">
+      <c r="F10" s="9">
+        <v>0</v>
+      </c>
+      <c r="G10" s="9">
+        <v>0</v>
+      </c>
+      <c r="H10" s="9">
         <v>89.009299999999996</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I10" s="9">
         <v>87.829099999999997</v>
       </c>
-      <c r="J10" s="10">
+      <c r="J10" s="9">
         <v>0.99419999999999997</v>
       </c>
-      <c r="K10" s="10">
+      <c r="K10" s="9">
         <v>0.9536</v>
       </c>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
-      <c r="N10" s="10"/>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="9"/>
       <c r="O10" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="S10" s="9">
+      <c r="S10" s="8">
         <v>102</v>
       </c>
-      <c r="T10" s="10"/>
+      <c r="T10" s="9"/>
     </row>
     <row r="11" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">

</xml_diff>

<commit_message>
Add f_tensor function value tests to all test scripts
</commit_message>
<xml_diff>
--- a/examples/ExpectedOutput/ExpectedOutput.xlsx
+++ b/examples/ExpectedOutput/ExpectedOutput.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roelv\Documents\GitHub\Refactor_experiment\examples\ExpectedOutput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69B4D063-A29F-4440-B5F9-DB6688916CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5590790A-4EDF-4B54-B523-EACCF905226C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{88699A24-984F-4F2B-A742-AB6C3C8D87BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="25">
   <si>
     <t>Example script number</t>
   </si>
@@ -806,49 +806,49 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:20" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+    <row r="7" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="7">
         <v>4</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="7">
         <v>3.5564999999999999E-2</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="7">
         <v>3.5564999999999999E-2</v>
       </c>
-      <c r="E7" s="9">
-        <v>0</v>
-      </c>
-      <c r="F7" s="9">
-        <v>0</v>
-      </c>
-      <c r="G7" s="9">
-        <v>0</v>
-      </c>
-      <c r="I7" s="9">
+      <c r="E7" s="7">
+        <v>0</v>
+      </c>
+      <c r="F7" s="7">
+        <v>0</v>
+      </c>
+      <c r="G7" s="7">
+        <v>0</v>
+      </c>
+      <c r="I7" s="7">
         <v>96.4435</v>
       </c>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9">
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7">
         <v>1</v>
       </c>
-      <c r="M7" s="9">
+      <c r="M7" s="7">
         <v>0.99529999999999996</v>
       </c>
-      <c r="N7" s="9">
+      <c r="N7" s="7">
         <v>1</v>
       </c>
-      <c r="O7" s="8" t="s">
+      <c r="O7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="S7" s="8">
+      <c r="S7" s="6">
         <v>201</v>
       </c>
-      <c r="T7" s="9" t="s">
+      <c r="T7" s="7" t="s">
         <v>19</v>
       </c>
     </row>
@@ -989,13 +989,15 @@
       <c r="L10" s="9"/>
       <c r="M10" s="9"/>
       <c r="N10" s="9"/>
-      <c r="O10" s="5" t="s">
+      <c r="O10" s="8" t="s">
         <v>14</v>
       </c>
       <c r="S10" s="8">
         <v>102</v>
       </c>
-      <c r="T10" s="9"/>
+      <c r="T10" s="9" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="11" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">

</xml_diff>